<commit_message>
chore: update Job_Search_Tracker with latest test execution records
</commit_message>
<xml_diff>
--- a/Job_Search_Tracker.xlsx
+++ b/Job_Search_Tracker.xlsx
@@ -900,7 +900,7 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr"/>
@@ -918,7 +918,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>2026-10-15T09:20:33.702275</t>
+          <t>2026-10-18T09:32:14.009377</t>
         </is>
       </c>
       <c r="AI2" t="inlineStr">

</xml_diff>